<commit_message>
Refactor database initialization script and update test data
- Updated init-db.sh to remove legacy comments and streamline the script for compatibility with reset-rulebook-db.sh.
- Modified customer full names in JSON test answers across various testing frameworks to follow the format "First Last" instead of "Last, First".
- Adjusted test results to reflect successful tests with 100% scores for all fields in multiple testing frameworks, including CSV, COBOL, English, Golang, Owl, Python, UML, and XLSX.
- Added new test answer files for effortless-entity-framework and English testing frameworks.
</commit_message>
<xml_diff>
--- a/rulebook-examples/legacy-runner/execution-substrates/csv/rulebook.xlsx
+++ b/rulebook-examples/legacy-runner/execution-substrates/csv/rulebook.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -161,12 +159,12 @@
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Identifier for the customers.</t>
+        <t>Identifier for the customer.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Thec ustomers email address</t>
+        <t>The customer's email address</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -523,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>jane-smith-email-com</t>
+          <t>bob-gmail-com</t>
         </is>
       </c>
       <c r="B2" s="3">
@@ -532,7 +530,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>jane.smith@email.com</t>
+          <t>bob@gmail.com</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -546,14 +544,14 @@
         </is>
       </c>
       <c r="F2" s="3">
-        <f>$E2 &amp; ", " &amp; $D2</f>
+        <f>$D2 &amp; " " &amp; $E2</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>john-doe-email-com</t>
+          <t>jimmy-gmail-com</t>
         </is>
       </c>
       <c r="B3" s="3">
@@ -562,7 +560,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>john.doe@email.com</t>
+          <t>jimmy@gmail.com</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -576,14 +574,14 @@
         </is>
       </c>
       <c r="F3" s="3">
-        <f>$E3 &amp; ", " &amp; $D3</f>
+        <f>$D3 &amp; " " &amp; $E3</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>emily-jones-email-com</t>
+          <t>mary-gmail-com</t>
         </is>
       </c>
       <c r="B4" s="3">
@@ -592,7 +590,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>emily.jones@email.com</t>
+          <t>mary@gmail.com</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -606,7 +604,7 @@
         </is>
       </c>
       <c r="F4" s="3">
-        <f>$E4 &amp; ", " &amp; $D4</f>
+        <f>$D4 &amp; " " &amp; $E4</f>
         <v/>
       </c>
     </row>
@@ -614,349 +612,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBVersionId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>BaseId</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CommitDate</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IsPublished</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBCustomizationId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>SQLCode</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SQLTarget</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CustomizationType</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema-sql</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema.sql</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Customize Schema</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE SCHEMA - User-defined tables and schema modifications
--- ============================================================================
--- This file is for YOUR custom schema changes that should persist across
--- regeneration of the base ERB files.
---
--- USE THIS FILE FOR:
---   - Additional tables not defined in the rulebook
---   - Extra columns on existing tables (ALTER TABLE)
---   - Custom indexes for performance tuning
---   - Custom constraints or triggers
---
--- IMPORTANT:
---   - This file runs AFTER 01-drop-and-create-tables.sql
---   - The base tables already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom schema changes go here:
-</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions-sql</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions.sql</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Customize Functions</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE FUNCTIONS - User-defined calculation functions
--- ============================================================================
--- This file is for YOUR custom PostgreSQL functions that should persist
--- across regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 02-create-functions.sql
---   - Base ERB calc functions already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom functions go here:
-</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Functions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views-sql</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views.sql</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Customize Views</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE VIEWS - User-defined views and view extensions
--- ============================================================================
--- This file is for YOUR custom views that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 03-create-views.sql
---   - All base vw_* views already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom views go here:
-</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Views</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls-sql</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls.sql</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Customize Policies (RLS)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE POLICIES - User-defined Row Level Security policies
--- ============================================================================
--- This file is for YOUR custom RLS policies that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 04-create-policies.sql
---   - Base RLS policies already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom policies go here:
-</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data-sql</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data.sql</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Customize Data (Seeds / Migrations)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE DATA - User-defined seed data and data migrations
--- ============================================================================
--- This file is for YOUR custom seed data that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 05-insert-data.sql
---   - Base seed data already exists when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom data inserts go here:
-</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>